<commit_message>
unidades passam a usar bloco configurável
</commit_message>
<xml_diff>
--- a/apps/web/e2e/fixtures/moradores.xlsx
+++ b/apps/web/e2e/fixtures/moradores.xlsx
@@ -8,9 +8,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
-    <t>Torre</t>
+    <t>Bloco</t>
   </si>
   <si>
     <t>Unidade</t>
@@ -57,6 +57,12 @@
   <si>
     <t>(11) 98877-1020</t>
   </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
 </sst>
 </file>
 
@@ -84,8 +90,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2">
-        <v>1</v>
+      <c r="A2" t="s">
+        <v>16</v>
       </c>
       <c r="B2">
         <v>12</v>
@@ -104,8 +110,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3">
-        <v>1</v>
+      <c r="A3" t="s">
+        <v>16</v>
       </c>
       <c r="B3">
         <v>12</v>
@@ -124,8 +130,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4">
-        <v>2</v>
+      <c r="A4" t="s">
+        <v>17</v>
       </c>
       <c r="B4">
         <v>104</v>

</xml_diff>